<commit_message>
update account book 10/06
</commit_message>
<xml_diff>
--- a/ledger/東京科学大学_UniLab_収支簿.xlsx
+++ b/ledger/東京科学大学_UniLab_収支簿.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ibuki_ono\Documents\hobby\rogiken\UniLab\ATOM\money\ChallengeATOM_AccountBook\ledger\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{302E0C0A-D671-45D6-A23F-2A768E93AE9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDA56508-D5B9-4773-8590-91F1D2CC9257}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{75F665F8-64B8-479F-B0B6-4F1BD8BBEF60}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{75F665F8-64B8-479F-B0B6-4F1BD8BBEF60}"/>
   </bookViews>
   <sheets>
     <sheet name="book" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="57">
   <si>
     <t>日付</t>
   </si>
@@ -91,95 +91,106 @@
     <t>OCS</t>
   </si>
   <si>
-    <t>物品費</t>
-    <phoneticPr fontId="18"/>
+    <t>口座入金</t>
+  </si>
+  <si>
+    <t>口座出金</t>
+  </si>
+  <si>
+    <t>未払金（クレジットカード支払い）</t>
+  </si>
+  <si>
+    <t>入金</t>
+  </si>
+  <si>
+    <t>開発助成金入金分</t>
   </si>
   <si>
     <t>クランプ、USBケーブル</t>
-    <phoneticPr fontId="18"/>
   </si>
   <si>
     <t>ロボットアームを動作補助として</t>
-    <rPh sb="8" eb="10">
-      <t>ドウサ</t>
-    </rPh>
-    <rPh sb="10" eb="12">
-      <t>ホジョ</t>
-    </rPh>
-    <phoneticPr fontId="18"/>
-  </si>
-  <si>
-    <t>Amazon</t>
-    <phoneticPr fontId="18"/>
   </si>
   <si>
     <t>ロボット用コントローラ</t>
-    <rPh sb="4" eb="5">
-      <t>ヨウ</t>
-    </rPh>
-    <phoneticPr fontId="18"/>
   </si>
   <si>
     <t>ロボットアーム</t>
-    <phoneticPr fontId="18"/>
   </si>
   <si>
     <t>Hardoff</t>
-    <phoneticPr fontId="18"/>
-  </si>
-  <si>
-    <t>口座入金</t>
-    <rPh sb="0" eb="2">
-      <t>コウザ</t>
-    </rPh>
-    <rPh sb="2" eb="4">
-      <t>ニュウキン</t>
-    </rPh>
-    <phoneticPr fontId="18"/>
-  </si>
-  <si>
-    <t>口座出金</t>
-    <rPh sb="0" eb="2">
-      <t>コウザ</t>
-    </rPh>
-    <rPh sb="2" eb="4">
-      <t>シュツキン</t>
-    </rPh>
-    <phoneticPr fontId="18"/>
-  </si>
-  <si>
-    <t>未払金（クレジットカード支払い）</t>
-    <rPh sb="0" eb="2">
-      <t>ミバラ</t>
-    </rPh>
-    <rPh sb="2" eb="3">
-      <t>キン</t>
-    </rPh>
-    <rPh sb="12" eb="14">
-      <t>シハラ</t>
-    </rPh>
-    <phoneticPr fontId="18"/>
-  </si>
-  <si>
-    <t>入金</t>
-    <rPh sb="0" eb="2">
-      <t>ニュウキン</t>
-    </rPh>
-    <phoneticPr fontId="18"/>
-  </si>
-  <si>
-    <t>開発助成金入金分</t>
-    <rPh sb="0" eb="5">
-      <t>カイハツジョセイキン</t>
-    </rPh>
-    <rPh sb="5" eb="8">
-      <t>ニュウキンブン</t>
-    </rPh>
-    <phoneticPr fontId="18"/>
-  </si>
-  <si>
-    <t>2_1</t>
-    <phoneticPr fontId="18"/>
+  </si>
+  <si>
+    <t>出金</t>
+  </si>
+  <si>
+    <t>未払金の回収</t>
+  </si>
+  <si>
+    <t>ロボット制御用自作基板</t>
+  </si>
+  <si>
+    <t>ロボットアームおよび車輪制御用として</t>
+  </si>
+  <si>
+    <t>JLCPCB</t>
+  </si>
+  <si>
+    <t>基板輸入関税</t>
+  </si>
+  <si>
+    <t>DHL</t>
+  </si>
+  <si>
+    <t>ロボット用センサ</t>
+  </si>
+  <si>
+    <t>ロボットの自動化を実現するため</t>
+  </si>
+  <si>
+    <t>光響</t>
+  </si>
+  <si>
+    <t>アルミフレーム</t>
+  </si>
+  <si>
+    <t>ロボットの構造体として</t>
+  </si>
+  <si>
+    <t>マイク</t>
+  </si>
+  <si>
+    <t>音源の方向推定の用途として</t>
+  </si>
+  <si>
+    <t>marutsu</t>
+  </si>
+  <si>
+    <t>スイッチングハブ</t>
+  </si>
+  <si>
+    <t>LANポート拡張用として</t>
+  </si>
+  <si>
+    <t>ポータブル電源</t>
+  </si>
+  <si>
+    <t>ロボット用の電源として</t>
+  </si>
+  <si>
+    <t>EcoFlow</t>
+  </si>
+  <si>
+    <t>DCジャック拡張</t>
+  </si>
+  <si>
+    <t>ロボットの非常停止用途として</t>
+  </si>
+  <si>
+    <t>ロボット用電源リレー</t>
+  </si>
+  <si>
+    <t>AliExpress</t>
   </si>
 </sst>
 </file>
@@ -788,8 +799,8 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -1166,7 +1177,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0383DCA2-8BAD-4AAF-AA73-51EE84FFE068}">
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J22"/>
   <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="10.19921875" style="1" bestFit="1" customWidth="1"/>
@@ -1181,7 +1192,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
@@ -1193,22 +1204,22 @@
       <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>32</v>
+      <c r="F1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G1" t="s">
+        <v>24</v>
+      </c>
+      <c r="H1" t="s">
+        <v>25</v>
       </c>
       <c r="I1" t="s">
         <v>5</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="J1" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1225,16 +1236,18 @@
       <c r="D2" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="4">
         <v>7612</v>
       </c>
-      <c r="H2" s="2">
+      <c r="F2"/>
+      <c r="G2"/>
+      <c r="H2" s="4">
         <v>7612</v>
       </c>
       <c r="I2" t="s">
         <v>10</v>
       </c>
-      <c r="J2" s="3">
+      <c r="J2">
         <v>1</v>
       </c>
     </row>
@@ -1251,16 +1264,18 @@
       <c r="D3" t="s">
         <v>12</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="4">
         <v>289596</v>
       </c>
-      <c r="H3" s="2">
+      <c r="F3"/>
+      <c r="G3"/>
+      <c r="H3" s="4">
         <v>289596</v>
       </c>
       <c r="I3" t="s">
         <v>13</v>
       </c>
-      <c r="J3" s="3">
+      <c r="J3">
         <v>2</v>
       </c>
     </row>
@@ -1277,16 +1292,18 @@
       <c r="D4" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="4">
         <v>285100</v>
       </c>
-      <c r="H4" s="2">
+      <c r="F4"/>
+      <c r="G4"/>
+      <c r="H4" s="4">
         <v>285100</v>
       </c>
       <c r="I4" t="s">
         <v>16</v>
       </c>
-      <c r="J4" s="3">
+      <c r="J4">
         <v>3</v>
       </c>
     </row>
@@ -1295,17 +1312,20 @@
         <v>46251</v>
       </c>
       <c r="B5" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="C5" t="s">
-        <v>34</v>
-      </c>
-      <c r="E5" s="2">
+        <v>27</v>
+      </c>
+      <c r="E5" s="4">
         <v>1000000</v>
       </c>
-      <c r="F5" s="2">
+      <c r="F5">
         <v>1000000</v>
       </c>
+      <c r="G5"/>
+      <c r="H5"/>
+      <c r="J5"/>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A6" s="1">
@@ -1320,16 +1340,18 @@
       <c r="D6" t="s">
         <v>18</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="4">
         <v>16829</v>
       </c>
-      <c r="H6" s="2">
+      <c r="F6"/>
+      <c r="G6"/>
+      <c r="H6" s="4">
         <v>16829</v>
       </c>
       <c r="I6" t="s">
         <v>19</v>
       </c>
-      <c r="J6" s="3">
+      <c r="J6">
         <v>4</v>
       </c>
     </row>
@@ -1346,17 +1368,19 @@
       <c r="D7" t="s">
         <v>21</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="4">
         <v>29050</v>
       </c>
-      <c r="G7" s="2">
+      <c r="F7"/>
+      <c r="G7" s="4">
         <v>29050</v>
       </c>
+      <c r="H7"/>
       <c r="I7" t="s">
         <v>22</v>
       </c>
-      <c r="J7" s="3" t="s">
-        <v>35</v>
+      <c r="J7">
+        <v>3</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.45">
@@ -1364,24 +1388,26 @@
         <v>46263</v>
       </c>
       <c r="B8" t="s">
-        <v>23</v>
+        <v>7</v>
       </c>
       <c r="C8" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="D8" t="s">
-        <v>25</v>
-      </c>
-      <c r="E8" s="2">
+        <v>29</v>
+      </c>
+      <c r="E8" s="4">
         <v>1762</v>
       </c>
-      <c r="H8" s="2">
+      <c r="F8"/>
+      <c r="G8"/>
+      <c r="H8" s="4">
         <v>1762</v>
       </c>
       <c r="I8" t="s">
-        <v>26</v>
-      </c>
-      <c r="J8" s="3">
+        <v>19</v>
+      </c>
+      <c r="J8">
         <v>5</v>
       </c>
     </row>
@@ -1390,26 +1416,340 @@
         <v>46262</v>
       </c>
       <c r="B9" t="s">
-        <v>23</v>
+        <v>7</v>
       </c>
       <c r="C9" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="D9" t="s">
-        <v>28</v>
-      </c>
-      <c r="E9" s="2">
+        <v>31</v>
+      </c>
+      <c r="E9" s="4">
         <v>3300</v>
       </c>
-      <c r="H9" s="2">
+      <c r="F9"/>
+      <c r="G9"/>
+      <c r="H9" s="4">
         <v>3300</v>
       </c>
       <c r="I9" t="s">
-        <v>29</v>
-      </c>
-      <c r="J9" s="3">
+        <v>32</v>
+      </c>
+      <c r="J9">
         <v>6</v>
       </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A10" s="1">
+        <v>46275</v>
+      </c>
+      <c r="B10" t="s">
+        <v>33</v>
+      </c>
+      <c r="C10" t="s">
+        <v>34</v>
+      </c>
+      <c r="E10" s="4">
+        <v>582308</v>
+      </c>
+      <c r="F10"/>
+      <c r="G10">
+        <v>582308</v>
+      </c>
+      <c r="H10"/>
+      <c r="J10"/>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A11" s="1">
+        <v>46275</v>
+      </c>
+      <c r="B11" t="s">
+        <v>7</v>
+      </c>
+      <c r="C11" t="s">
+        <v>35</v>
+      </c>
+      <c r="D11" t="s">
+        <v>36</v>
+      </c>
+      <c r="E11" s="4">
+        <v>17738</v>
+      </c>
+      <c r="F11"/>
+      <c r="G11"/>
+      <c r="H11" s="4">
+        <v>17738</v>
+      </c>
+      <c r="I11" t="s">
+        <v>37</v>
+      </c>
+      <c r="J11">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A12" s="1">
+        <v>46276</v>
+      </c>
+      <c r="B12" t="s">
+        <v>7</v>
+      </c>
+      <c r="C12" t="s">
+        <v>38</v>
+      </c>
+      <c r="D12" t="s">
+        <v>21</v>
+      </c>
+      <c r="E12" s="4">
+        <v>3900</v>
+      </c>
+      <c r="F12"/>
+      <c r="G12">
+        <v>3900</v>
+      </c>
+      <c r="H12"/>
+      <c r="I12" t="s">
+        <v>39</v>
+      </c>
+      <c r="J12">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A13" s="1">
+        <v>46279</v>
+      </c>
+      <c r="B13" t="s">
+        <v>7</v>
+      </c>
+      <c r="C13" t="s">
+        <v>40</v>
+      </c>
+      <c r="D13" t="s">
+        <v>41</v>
+      </c>
+      <c r="E13" s="4">
+        <v>88550</v>
+      </c>
+      <c r="F13"/>
+      <c r="G13" s="4">
+        <v>88550</v>
+      </c>
+      <c r="H13"/>
+      <c r="I13" t="s">
+        <v>42</v>
+      </c>
+      <c r="J13">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A14" s="1">
+        <v>46283</v>
+      </c>
+      <c r="B14" t="s">
+        <v>7</v>
+      </c>
+      <c r="C14" t="s">
+        <v>43</v>
+      </c>
+      <c r="D14" t="s">
+        <v>44</v>
+      </c>
+      <c r="E14" s="4">
+        <v>18990</v>
+      </c>
+      <c r="F14"/>
+      <c r="G14"/>
+      <c r="H14">
+        <v>18990</v>
+      </c>
+      <c r="I14" t="s">
+        <v>10</v>
+      </c>
+      <c r="J14">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A15" s="1">
+        <v>46287</v>
+      </c>
+      <c r="B15" t="s">
+        <v>7</v>
+      </c>
+      <c r="C15" t="s">
+        <v>45</v>
+      </c>
+      <c r="D15" t="s">
+        <v>46</v>
+      </c>
+      <c r="E15" s="4">
+        <v>10063</v>
+      </c>
+      <c r="F15"/>
+      <c r="G15">
+        <v>10063</v>
+      </c>
+      <c r="H15"/>
+      <c r="I15" t="s">
+        <v>47</v>
+      </c>
+      <c r="J15">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A16" s="1">
+        <v>46293</v>
+      </c>
+      <c r="B16" t="s">
+        <v>7</v>
+      </c>
+      <c r="C16" t="s">
+        <v>48</v>
+      </c>
+      <c r="D16" t="s">
+        <v>49</v>
+      </c>
+      <c r="E16" s="4">
+        <v>7400</v>
+      </c>
+      <c r="F16"/>
+      <c r="G16"/>
+      <c r="H16">
+        <v>7400</v>
+      </c>
+      <c r="I16" t="s">
+        <v>19</v>
+      </c>
+      <c r="J16">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A17" s="1">
+        <v>46293</v>
+      </c>
+      <c r="B17" t="s">
+        <v>7</v>
+      </c>
+      <c r="C17" t="s">
+        <v>50</v>
+      </c>
+      <c r="D17" t="s">
+        <v>51</v>
+      </c>
+      <c r="E17" s="4">
+        <v>40000</v>
+      </c>
+      <c r="F17"/>
+      <c r="G17"/>
+      <c r="H17">
+        <v>40000</v>
+      </c>
+      <c r="I17" t="s">
+        <v>52</v>
+      </c>
+      <c r="J17">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A18" s="1">
+        <v>46294</v>
+      </c>
+      <c r="B18" t="s">
+        <v>7</v>
+      </c>
+      <c r="C18" t="s">
+        <v>53</v>
+      </c>
+      <c r="D18" t="s">
+        <v>51</v>
+      </c>
+      <c r="E18">
+        <v>799</v>
+      </c>
+      <c r="F18"/>
+      <c r="G18"/>
+      <c r="H18">
+        <v>799</v>
+      </c>
+      <c r="I18" t="s">
+        <v>19</v>
+      </c>
+      <c r="J18">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A19" s="1">
+        <v>46296</v>
+      </c>
+      <c r="B19" t="s">
+        <v>7</v>
+      </c>
+      <c r="C19" t="s">
+        <v>35</v>
+      </c>
+      <c r="D19" t="s">
+        <v>54</v>
+      </c>
+      <c r="E19" s="4">
+        <v>6254</v>
+      </c>
+      <c r="F19"/>
+      <c r="G19"/>
+      <c r="H19"/>
+      <c r="I19" t="s">
+        <v>37</v>
+      </c>
+      <c r="J19">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A20" s="1">
+        <v>46292</v>
+      </c>
+      <c r="B20" t="s">
+        <v>7</v>
+      </c>
+      <c r="C20" t="s">
+        <v>55</v>
+      </c>
+      <c r="D20" t="s">
+        <v>54</v>
+      </c>
+      <c r="E20" s="4">
+        <v>5714</v>
+      </c>
+      <c r="F20"/>
+      <c r="G20"/>
+      <c r="H20"/>
+      <c r="I20" t="s">
+        <v>56</v>
+      </c>
+      <c r="J20">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A21"/>
+      <c r="E21"/>
+      <c r="F21"/>
+      <c r="G21"/>
+      <c r="H21"/>
+      <c r="J21"/>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A22"/>
+      <c r="E22"/>
+      <c r="F22"/>
+      <c r="G22"/>
+      <c r="H22"/>
+      <c r="J22"/>
     </row>
   </sheetData>
   <phoneticPr fontId="18"/>

</xml_diff>

<commit_message>
update ledger and evidence
</commit_message>
<xml_diff>
--- a/ledger/東京科学大学_UniLab_収支簿.xlsx
+++ b/ledger/東京科学大学_UniLab_収支簿.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ibuki_ono\Documents\hobby\rogiken\UniLab\ATOM\money\ChallengeATOM_AccountBook\ledger\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDA56508-D5B9-4773-8590-91F1D2CC9257}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41BF97B4-DE2D-4820-B1C3-22BA3C78A7FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{75F665F8-64B8-479F-B0B6-4F1BD8BBEF60}"/>
   </bookViews>
@@ -20,10 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="57">
-  <si>
-    <t>日付</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="63">
   <si>
     <t>費目</t>
   </si>
@@ -191,6 +188,27 @@
   </si>
   <si>
     <t>AliExpress</t>
+  </si>
+  <si>
+    <t>購入日</t>
+  </si>
+  <si>
+    <t>LEDライトバー</t>
+  </si>
+  <si>
+    <t>ロボットの警告灯として</t>
+  </si>
+  <si>
+    <t>カメラ</t>
+  </si>
+  <si>
+    <t>ロボット外部、植物監視用途として</t>
+  </si>
+  <si>
+    <t>GNSSセンサ</t>
+  </si>
+  <si>
+    <t>ロボット自己位置推定用途として</t>
   </si>
 </sst>
 </file>
@@ -1177,7 +1195,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0383DCA2-8BAD-4AAF-AA73-51EE84FFE068}">
-  <dimension ref="A1:J22"/>
+  <dimension ref="A1:J23"/>
   <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="10.19921875" style="1" bestFit="1" customWidth="1"/>
@@ -1193,34 +1211,34 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H1" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
-        <v>23</v>
-      </c>
-      <c r="G1" t="s">
-        <v>24</v>
-      </c>
-      <c r="H1" t="s">
-        <v>25</v>
-      </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>5</v>
-      </c>
-      <c r="J1" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.45">
@@ -1228,13 +1246,13 @@
         <v>46228</v>
       </c>
       <c r="B2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>8</v>
-      </c>
-      <c r="D2" t="s">
-        <v>9</v>
       </c>
       <c r="E2" s="4">
         <v>7612</v>
@@ -1245,7 +1263,7 @@
         <v>7612</v>
       </c>
       <c r="I2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1256,13 +1274,13 @@
         <v>46237</v>
       </c>
       <c r="B3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" t="s">
         <v>11</v>
-      </c>
-      <c r="D3" t="s">
-        <v>12</v>
       </c>
       <c r="E3" s="4">
         <v>289596</v>
@@ -1273,7 +1291,7 @@
         <v>289596</v>
       </c>
       <c r="I3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1284,13 +1302,13 @@
         <v>46237</v>
       </c>
       <c r="B4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" t="s">
         <v>14</v>
-      </c>
-      <c r="D4" t="s">
-        <v>15</v>
       </c>
       <c r="E4" s="4">
         <v>285100</v>
@@ -1301,7 +1319,7 @@
         <v>285100</v>
       </c>
       <c r="I4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1312,10 +1330,10 @@
         <v>46251</v>
       </c>
       <c r="B5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C5" t="s">
         <v>26</v>
-      </c>
-      <c r="C5" t="s">
-        <v>27</v>
       </c>
       <c r="E5" s="4">
         <v>1000000</v>
@@ -1332,13 +1350,13 @@
         <v>46258</v>
       </c>
       <c r="B6" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C6" t="s">
+        <v>16</v>
+      </c>
+      <c r="D6" t="s">
         <v>17</v>
-      </c>
-      <c r="D6" t="s">
-        <v>18</v>
       </c>
       <c r="E6" s="4">
         <v>16829</v>
@@ -1349,7 +1367,7 @@
         <v>16829</v>
       </c>
       <c r="I6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J6">
         <v>4</v>
@@ -1360,13 +1378,13 @@
         <v>46261</v>
       </c>
       <c r="B7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C7" t="s">
+        <v>19</v>
+      </c>
+      <c r="D7" t="s">
         <v>20</v>
-      </c>
-      <c r="D7" t="s">
-        <v>21</v>
       </c>
       <c r="E7" s="4">
         <v>29050</v>
@@ -1377,7 +1395,7 @@
       </c>
       <c r="H7"/>
       <c r="I7" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="J7">
         <v>3</v>
@@ -1388,13 +1406,13 @@
         <v>46263</v>
       </c>
       <c r="B8" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C8" t="s">
+        <v>27</v>
+      </c>
+      <c r="D8" t="s">
         <v>28</v>
-      </c>
-      <c r="D8" t="s">
-        <v>29</v>
       </c>
       <c r="E8" s="4">
         <v>1762</v>
@@ -1405,7 +1423,7 @@
         <v>1762</v>
       </c>
       <c r="I8" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J8">
         <v>5</v>
@@ -1416,13 +1434,13 @@
         <v>46262</v>
       </c>
       <c r="B9" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C9" t="s">
+        <v>29</v>
+      </c>
+      <c r="D9" t="s">
         <v>30</v>
-      </c>
-      <c r="D9" t="s">
-        <v>31</v>
       </c>
       <c r="E9" s="4">
         <v>3300</v>
@@ -1433,7 +1451,7 @@
         <v>3300</v>
       </c>
       <c r="I9" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="J9">
         <v>6</v>
@@ -1444,10 +1462,10 @@
         <v>46275</v>
       </c>
       <c r="B10" t="s">
+        <v>32</v>
+      </c>
+      <c r="C10" t="s">
         <v>33</v>
-      </c>
-      <c r="C10" t="s">
-        <v>34</v>
       </c>
       <c r="E10" s="4">
         <v>582308</v>
@@ -1464,13 +1482,13 @@
         <v>46275</v>
       </c>
       <c r="B11" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C11" t="s">
+        <v>34</v>
+      </c>
+      <c r="D11" t="s">
         <v>35</v>
-      </c>
-      <c r="D11" t="s">
-        <v>36</v>
       </c>
       <c r="E11" s="4">
         <v>17738</v>
@@ -1481,7 +1499,7 @@
         <v>17738</v>
       </c>
       <c r="I11" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="J11">
         <v>7</v>
@@ -1492,13 +1510,13 @@
         <v>46276</v>
       </c>
       <c r="B12" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C12" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E12" s="4">
         <v>3900</v>
@@ -1509,7 +1527,7 @@
       </c>
       <c r="H12"/>
       <c r="I12" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="J12">
         <v>7</v>
@@ -1520,13 +1538,13 @@
         <v>46279</v>
       </c>
       <c r="B13" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C13" t="s">
+        <v>39</v>
+      </c>
+      <c r="D13" t="s">
         <v>40</v>
-      </c>
-      <c r="D13" t="s">
-        <v>41</v>
       </c>
       <c r="E13" s="4">
         <v>88550</v>
@@ -1537,7 +1555,7 @@
       </c>
       <c r="H13"/>
       <c r="I13" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J13">
         <v>8</v>
@@ -1548,13 +1566,13 @@
         <v>46283</v>
       </c>
       <c r="B14" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C14" t="s">
+        <v>42</v>
+      </c>
+      <c r="D14" t="s">
         <v>43</v>
-      </c>
-      <c r="D14" t="s">
-        <v>44</v>
       </c>
       <c r="E14" s="4">
         <v>18990</v>
@@ -1565,7 +1583,7 @@
         <v>18990</v>
       </c>
       <c r="I14" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="J14">
         <v>10</v>
@@ -1576,13 +1594,13 @@
         <v>46287</v>
       </c>
       <c r="B15" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C15" t="s">
+        <v>44</v>
+      </c>
+      <c r="D15" t="s">
         <v>45</v>
-      </c>
-      <c r="D15" t="s">
-        <v>46</v>
       </c>
       <c r="E15" s="4">
         <v>10063</v>
@@ -1593,7 +1611,7 @@
       </c>
       <c r="H15"/>
       <c r="I15" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="J15">
         <v>9</v>
@@ -1604,13 +1622,13 @@
         <v>46293</v>
       </c>
       <c r="B16" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C16" t="s">
+        <v>47</v>
+      </c>
+      <c r="D16" t="s">
         <v>48</v>
-      </c>
-      <c r="D16" t="s">
-        <v>49</v>
       </c>
       <c r="E16" s="4">
         <v>7400</v>
@@ -1621,7 +1639,7 @@
         <v>7400</v>
       </c>
       <c r="I16" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J16">
         <v>11</v>
@@ -1632,13 +1650,13 @@
         <v>46293</v>
       </c>
       <c r="B17" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C17" t="s">
+        <v>49</v>
+      </c>
+      <c r="D17" t="s">
         <v>50</v>
-      </c>
-      <c r="D17" t="s">
-        <v>51</v>
       </c>
       <c r="E17" s="4">
         <v>40000</v>
@@ -1649,7 +1667,7 @@
         <v>40000</v>
       </c>
       <c r="I17" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="J17">
         <v>13</v>
@@ -1660,13 +1678,13 @@
         <v>46294</v>
       </c>
       <c r="B18" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C18" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D18" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E18">
         <v>799</v>
@@ -1677,7 +1695,7 @@
         <v>799</v>
       </c>
       <c r="I18" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J18">
         <v>12</v>
@@ -1688,22 +1706,24 @@
         <v>46296</v>
       </c>
       <c r="B19" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C19" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D19" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E19" s="4">
-        <v>6254</v>
+        <v>6494</v>
       </c>
       <c r="F19"/>
       <c r="G19"/>
-      <c r="H19"/>
+      <c r="H19">
+        <v>6494</v>
+      </c>
       <c r="I19" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="J19">
         <v>14</v>
@@ -1714,45 +1734,116 @@
         <v>46292</v>
       </c>
       <c r="B20" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C20" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D20" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E20" s="4">
         <v>5714</v>
       </c>
       <c r="F20"/>
       <c r="G20"/>
-      <c r="H20"/>
+      <c r="H20">
+        <v>5714</v>
+      </c>
       <c r="I20" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="J20">
         <v>15</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A21"/>
-      <c r="E21"/>
+      <c r="A21" s="1">
+        <v>46286</v>
+      </c>
+      <c r="B21" t="s">
+        <v>6</v>
+      </c>
+      <c r="C21" t="s">
+        <v>57</v>
+      </c>
+      <c r="D21" t="s">
+        <v>58</v>
+      </c>
+      <c r="E21" s="4">
+        <v>4477</v>
+      </c>
       <c r="F21"/>
       <c r="G21"/>
-      <c r="H21"/>
-      <c r="J21"/>
+      <c r="H21">
+        <v>4477</v>
+      </c>
+      <c r="I21" t="s">
+        <v>55</v>
+      </c>
+      <c r="J21">
+        <v>18</v>
+      </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A22"/>
-      <c r="E22"/>
+      <c r="A22" s="1">
+        <v>46287</v>
+      </c>
+      <c r="B22" t="s">
+        <v>6</v>
+      </c>
+      <c r="C22" t="s">
+        <v>59</v>
+      </c>
+      <c r="D22" t="s">
+        <v>60</v>
+      </c>
+      <c r="E22" s="4">
+        <v>16435</v>
+      </c>
       <c r="F22"/>
       <c r="G22"/>
-      <c r="H22"/>
-      <c r="J22"/>
+      <c r="H22">
+        <v>16436</v>
+      </c>
+      <c r="I22" t="s">
+        <v>55</v>
+      </c>
+      <c r="J22">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A23" s="1">
+        <v>46287</v>
+      </c>
+      <c r="B23" t="s">
+        <v>6</v>
+      </c>
+      <c r="C23" t="s">
+        <v>61</v>
+      </c>
+      <c r="D23" t="s">
+        <v>62</v>
+      </c>
+      <c r="E23" s="4">
+        <v>11148</v>
+      </c>
+      <c r="F23"/>
+      <c r="G23"/>
+      <c r="H23">
+        <v>11148</v>
+      </c>
+      <c r="I23" t="s">
+        <v>55</v>
+      </c>
+      <c r="J23">
+        <v>17</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="18"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="landscape" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>